<commit_message>
fix: update user import template validations
</commit_message>
<xml_diff>
--- a/frontend/school-management/public/assets/templates/users.xlsx
+++ b/frontend/school-management/public/assets/templates/users.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bfe8d841f309e89/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lopey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E225A5BE-3438-48B4-960B-9AB93FB51BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B5F6D0-6D1B-402D-95EF-D0A7FF38F23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C9BCE194-0BE2-4C32-A2BF-E9BC0733A790}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$F$1:$F$2</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -103,13 +106,21 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="170" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="171" formatCode="0;[Red]0"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -132,10 +143,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -145,16 +157,18 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -560,9 +574,60 @@
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="C2" s="9"/>
       <c r="D2" s="4"/>
     </row>
   </sheetData>
+  <dataValidations count="16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{90E786B0-3990-4CB5-ABA8-1E83324A660D}">
+      <formula1>"hombre,mujer"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{835F3B96-65A2-40E4-8FA2-4C7F8A6A052C}">
+      <formula1>B1&lt;&gt;""</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Telefono invalido" error="Escribe un telefono de 10 digitos_x000a_" sqref="D1:D1048576" xr:uid="{0A099B91-BDC2-4AE5-90EF-5C4ED75E466F}">
+      <formula1>AND(D1&lt;&gt;"",LEN(D1)=10,ISNUMBER(--D1))</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha invalida" sqref="E1:E1048576" xr:uid="{C6B5F758-7EFB-45C9-A05B-9B69065DC722}">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="CURP invalida" sqref="G1:G1048576" xr:uid="{AC7BA965-3CC4-48FF-B1AD-C2D9B70777C9}">
+      <formula1>AND(G1&lt;&gt;"",LEN(G1)=18)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Codigo postal invalido" error="Introduce un código postal de 5 digitos_x000a_" sqref="K1:K1048576" xr:uid="{7E34AE19-A16B-43A7-B1D8-A29DC2114BB5}">
+      <formula1>AND(LEN(K1)=5,ISNUMBER(--K1))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L1048576" xr:uid="{461A9CEE-98C2-414D-B5E0-42CA24CFA310}">
+      <formula1>"O+,O-,A+,A-,B+,B-,AB+,AB-"</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1:M1048576" xr:uid="{AF6C92BB-9E47-4FDE-A9F1-991BA8955C62}">
+      <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N1:N1048576" xr:uid="{D0AC5E29-556E-4FBD-BF63-A9CEB4FC2F43}">
+      <formula1>"activo,baja,baja-temporal"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P1 P3:P1048576" xr:uid="{56229DCA-08F0-453F-9013-A5DBE0D68DDC}">
+      <formula1>"'=Y(P2&lt;&gt;"""";LARGO(P2)=30)"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q1:Q1048576" xr:uid="{2674E65F-5594-4876-A7DF-4CD39BEF2FED}">
+      <formula1>"1,2,3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R1:R1048576" xr:uid="{2F78EC6B-8805-4315-A47D-8A5DC25913BF}">
+      <formula1>AND(LEN(R1)=10)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O1:O1048576" xr:uid="{33D70B84-ED1A-42C8-9A38-189C65835183}">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Correo invalido" error="Ingresa un correo electrónico válido." sqref="C1:C1048576" xr:uid="{042008F7-21AD-42BA-BD93-470746CFA6DF}">
+      <formula1>AND(C1&lt;&gt;"",ISNUMBER(SEARCH("@",C1)),ISNUMBER(SEARCH(".",C1)))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:A1048576" xr:uid="{C1DDDF46-E92F-40F4-97DA-2E639031EEDF}">
+      <formula1>A1&lt;&gt;""</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2" xr:uid="{204F28D2-247E-4FCB-962F-46C0AAEB142E}">
+      <formula1>AND(LEN(P1)=30)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>